<commit_message>
updated caledar for Lab06
</commit_message>
<xml_diff>
--- a/CS320-Spring2024Calendar.xlsx
+++ b/CS320-Spring2024Calendar.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cygwin64\home\donha\cs320-spring2024\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4166887-8506-437A-B465-9E33C6DF1E4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45B2E61C-B30A-4DFE-94AD-D4A81EB362BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="368" yWindow="368" windowWidth="26264" windowHeight="15127" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="435" yWindow="570" windowWidth="25425" windowHeight="15128" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calendar-Sp24" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="79">
   <si>
     <t>Monday</t>
   </si>
@@ -251,11 +251,6 @@
   </si>
   <si>
     <t>A08: Team Report due Noon
-(Marmoset)</t>
-  </si>
-  <si>
-    <t>Lab 6: ORM
-due  Noon
 (Marmoset)</t>
   </si>
   <si>
@@ -548,10 +543,6 @@
     <t>Assign06: Team Problem Domain Analysis Submission Review</t>
   </si>
   <si>
-    <t>CS320: SW Engineering - Spring 2024 Schedule
-(as of 3-19-2024, subject to change)</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Lecture  15: ORM, Designing a Persistence Layer
 </t>
@@ -582,6 +573,28 @@
   <si>
     <t>A03: Team MS2
 50% Progress on Features w/fake data</t>
+  </si>
+  <si>
+    <t>CS320: SW Engineering - Spring 2024 Schedule
+(as of 3-29-2024, subject to change)</t>
+  </si>
+  <si>
+    <t>Lab 6: ORM
+due  Noon
+for 50% EC
+(Marmoset)</t>
+  </si>
+  <si>
+    <t>Lab 6: ORM
+due  Noon
+for 25% EC
+(Marmoset)</t>
+  </si>
+  <si>
+    <t>Lab 6: ORM
+due  Noon
+for full credit
+(Marmoset)</t>
   </si>
 </sst>
 </file>
@@ -1283,7 +1296,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="158">
+  <cellXfs count="159">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1687,50 +1700,68 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
@@ -1738,22 +1769,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2083,17 +2099,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="53.1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="135" t="s">
-        <v>73</v>
-      </c>
-      <c r="B1" s="136"/>
-      <c r="C1" s="136"/>
-      <c r="D1" s="136"/>
-      <c r="E1" s="136"/>
-      <c r="F1" s="136"/>
-      <c r="G1" s="136"/>
-      <c r="H1" s="136"/>
-      <c r="I1" s="137"/>
+      <c r="A1" s="152" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="153"/>
+      <c r="C1" s="153"/>
+      <c r="D1" s="153"/>
+      <c r="E1" s="153"/>
+      <c r="F1" s="153"/>
+      <c r="G1" s="153"/>
+      <c r="H1" s="153"/>
+      <c r="I1" s="154"/>
     </row>
     <row r="2" spans="1:18" s="2" customFormat="1" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A2" s="1" t="s">
@@ -2123,10 +2139,10 @@
       </c>
     </row>
     <row r="3" spans="1:18" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="140">
+      <c r="A3" s="144">
         <v>15</v>
       </c>
-      <c r="B3" s="149" t="s">
+      <c r="B3" s="139" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="66">
@@ -2158,8 +2174,8 @@
       </c>
     </row>
     <row r="4" spans="1:18" ht="75.400000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A4" s="139"/>
-      <c r="B4" s="150"/>
+      <c r="A4" s="148"/>
+      <c r="B4" s="156"/>
       <c r="C4" s="68" t="s">
         <v>7</v>
       </c>
@@ -2180,16 +2196,16 @@
       </c>
       <c r="G4" s="37"/>
       <c r="H4" s="36" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I4" s="40"/>
     </row>
     <row r="5" spans="1:18" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="139">
+      <c r="A5" s="148">
         <f>A3 - 1</f>
         <v>14</v>
       </c>
-      <c r="B5" s="144" t="s">
+      <c r="B5" s="141" t="s">
         <v>27</v>
       </c>
       <c r="C5" s="7">
@@ -2221,30 +2237,30 @@
       </c>
     </row>
     <row r="6" spans="1:18" ht="146.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A6" s="141"/>
-      <c r="B6" s="145"/>
+      <c r="A6" s="145"/>
+      <c r="B6" s="140"/>
       <c r="C6" s="116" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D6" s="121" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E6" s="56"/>
       <c r="F6" s="117" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G6" s="48"/>
       <c r="H6" s="47" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I6" s="104"/>
     </row>
     <row r="7" spans="1:18" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="142">
+      <c r="A7" s="149">
         <f>A5 - 1</f>
         <v>13</v>
       </c>
-      <c r="B7" s="146" t="s">
+      <c r="B7" s="136" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="38">
@@ -2277,30 +2293,30 @@
       </c>
     </row>
     <row r="8" spans="1:18" ht="99.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="143"/>
-      <c r="B8" s="147"/>
+      <c r="A8" s="142"/>
+      <c r="B8" s="138"/>
       <c r="C8" s="30" t="s">
         <v>40</v>
       </c>
       <c r="D8" s="47" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E8" s="10"/>
       <c r="F8" s="12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G8" s="27"/>
       <c r="H8" s="10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I8" s="126"/>
     </row>
     <row r="9" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="143">
+      <c r="A9" s="142">
         <f>A7 - 1</f>
         <v>12</v>
       </c>
-      <c r="B9" s="147"/>
+      <c r="B9" s="138"/>
       <c r="C9" s="14">
         <f>I7 + 1</f>
         <v>11</v>
@@ -2338,8 +2354,8 @@
       <c r="R9" s="110"/>
     </row>
     <row r="10" spans="1:18" ht="102.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="143"/>
-      <c r="B10" s="147"/>
+      <c r="A10" s="142"/>
+      <c r="B10" s="138"/>
       <c r="C10" s="125" t="s">
         <v>37</v>
       </c>
@@ -2347,14 +2363,14 @@
         <v>35</v>
       </c>
       <c r="E10" s="105" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G10" s="11"/>
       <c r="H10" s="10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I10" s="13"/>
       <c r="L10" s="25"/>
@@ -2366,11 +2382,11 @@
       <c r="R10" s="111"/>
     </row>
     <row r="11" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="143">
+      <c r="A11" s="142">
         <f>A9 -1</f>
         <v>11</v>
       </c>
-      <c r="B11" s="147"/>
+      <c r="B11" s="138"/>
       <c r="C11" s="17">
         <f>I9 + 1</f>
         <v>18</v>
@@ -2408,23 +2424,23 @@
       <c r="R11" s="110"/>
     </row>
     <row r="12" spans="1:18" ht="115.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A12" s="143"/>
-      <c r="B12" s="147"/>
+      <c r="A12" s="142"/>
+      <c r="B12" s="138"/>
       <c r="C12" s="30" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D12" s="12" t="s">
         <v>31</v>
       </c>
       <c r="E12" s="132" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F12" s="44" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G12" s="42"/>
       <c r="H12" s="128" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I12" s="77"/>
       <c r="L12" s="25"/>
@@ -2436,11 +2452,11 @@
       <c r="R12" s="111"/>
     </row>
     <row r="13" spans="1:18" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="143">
+      <c r="A13" s="142">
         <f xml:space="preserve"> A11 - 1</f>
         <v>10</v>
       </c>
-      <c r="B13" s="151" t="s">
+      <c r="B13" s="157" t="s">
         <v>28</v>
       </c>
       <c r="C13" s="17">
@@ -2479,13 +2495,13 @@
       <c r="R13" s="112"/>
     </row>
     <row r="14" spans="1:18" ht="100.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A14" s="148"/>
-      <c r="B14" s="152"/>
+      <c r="A14" s="143"/>
+      <c r="B14" s="137"/>
       <c r="C14" s="129" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D14" s="123" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E14" s="89"/>
       <c r="F14" s="122" t="s">
@@ -2509,11 +2525,11 @@
       <c r="R14" s="112"/>
     </row>
     <row r="15" spans="1:18" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="140">
+      <c r="A15" s="144">
         <f>A13 - 1</f>
         <v>9</v>
       </c>
-      <c r="B15" s="144" t="s">
+      <c r="B15" s="141" t="s">
         <v>12</v>
       </c>
       <c r="C15" s="66">
@@ -2546,13 +2562,13 @@
       </c>
     </row>
     <row r="16" spans="1:18" ht="103.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A16" s="141"/>
-      <c r="B16" s="145"/>
+      <c r="A16" s="145"/>
+      <c r="B16" s="140"/>
       <c r="C16" s="85" t="s">
         <v>32</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E16" s="63" t="s">
         <v>26</v>
@@ -2575,7 +2591,7 @@
 (all in-class)</v>
       </c>
       <c r="I16" s="133" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:18" ht="6.4" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
@@ -2597,13 +2613,13 @@
         <v>15</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F18" s="32" t="s">
         <v>16</v>
       </c>
       <c r="G18" s="120" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H18" s="33" t="s">
         <v>17</v>
@@ -2624,19 +2640,19 @@
       <c r="I19" s="112"/>
     </row>
     <row r="20" spans="1:18" ht="54" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A20" s="135" t="str">
+      <c r="A20" s="152" t="str">
         <f>A1</f>
         <v>CS320: SW Engineering - Spring 2024 Schedule
-(as of 3-19-2024, subject to change)</v>
-      </c>
-      <c r="B20" s="136"/>
-      <c r="C20" s="136"/>
-      <c r="D20" s="136"/>
-      <c r="E20" s="136"/>
-      <c r="F20" s="136"/>
-      <c r="G20" s="136"/>
-      <c r="H20" s="136"/>
-      <c r="I20" s="137"/>
+(as of 3-29-2024, subject to change)</v>
+      </c>
+      <c r="B20" s="153"/>
+      <c r="C20" s="153"/>
+      <c r="D20" s="153"/>
+      <c r="E20" s="153"/>
+      <c r="F20" s="153"/>
+      <c r="G20" s="153"/>
+      <c r="H20" s="153"/>
+      <c r="I20" s="154"/>
     </row>
     <row r="21" spans="1:18" s="2" customFormat="1" ht="17.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A21" s="1" t="str">
@@ -2674,11 +2690,11 @@
       </c>
     </row>
     <row r="22" spans="1:18" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="138">
+      <c r="A22" s="155">
         <f>A15-1</f>
         <v>8</v>
       </c>
-      <c r="B22" s="144" t="s">
+      <c r="B22" s="141" t="s">
         <v>12</v>
       </c>
       <c r="C22" s="93">
@@ -2718,15 +2734,15 @@
       <c r="R22" s="110"/>
     </row>
     <row r="23" spans="1:18" ht="67.150000000000006" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A23" s="139"/>
-      <c r="B23" s="144"/>
+      <c r="A23" s="148"/>
+      <c r="B23" s="141"/>
       <c r="C23" s="134"/>
       <c r="D23" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E23" s="54"/>
       <c r="F23" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G23" s="6"/>
       <c r="H23" s="22" t="s">
@@ -2742,11 +2758,11 @@
       <c r="R23" s="25"/>
     </row>
     <row r="24" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A24" s="139">
+      <c r="A24" s="148">
         <f>A22 - 1</f>
         <v>7</v>
       </c>
-      <c r="B24" s="144"/>
+      <c r="B24" s="141"/>
       <c r="C24" s="7">
         <f>I22 + 1</f>
         <v>17</v>
@@ -2784,8 +2800,8 @@
       <c r="R24" s="110"/>
     </row>
     <row r="25" spans="1:18" ht="124.15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="139"/>
-      <c r="B25" s="144"/>
+      <c r="A25" s="148"/>
+      <c r="B25" s="141"/>
       <c r="C25" s="109"/>
       <c r="D25" s="26" t="s">
         <v>23</v>
@@ -2795,8 +2811,8 @@
         <v>38</v>
       </c>
       <c r="G25" s="127"/>
-      <c r="H25" s="157" t="s">
-        <v>74</v>
+      <c r="H25" s="135" t="s">
+        <v>72</v>
       </c>
       <c r="I25" s="131"/>
       <c r="L25" s="25"/>
@@ -2808,11 +2824,11 @@
       <c r="R25" s="25"/>
     </row>
     <row r="26" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A26" s="139">
+      <c r="A26" s="148">
         <f>A24 - 1</f>
         <v>6</v>
       </c>
-      <c r="B26" s="144"/>
+      <c r="B26" s="141"/>
       <c r="C26" s="7">
         <f>I24 + 1</f>
         <v>24</v>
@@ -2850,20 +2866,20 @@
       <c r="R26" s="110"/>
     </row>
     <row r="27" spans="1:18" ht="68.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A27" s="141"/>
-      <c r="B27" s="145"/>
+      <c r="A27" s="145"/>
+      <c r="B27" s="140"/>
       <c r="C27" s="130" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D27" s="9" t="s">
         <v>20</v>
       </c>
       <c r="E27" s="54"/>
       <c r="F27" s="23" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="G27" s="124" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H27" s="71" t="s">
         <v>36</v>
@@ -2880,11 +2896,11 @@
       <c r="R27" s="25"/>
     </row>
     <row r="28" spans="1:18" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A28" s="142">
+      <c r="A28" s="149">
         <f>A26 -1</f>
         <v>5</v>
       </c>
-      <c r="B28" s="146" t="s">
+      <c r="B28" s="136" t="s">
         <v>33</v>
       </c>
       <c r="C28" s="99">
@@ -2916,8 +2932,8 @@
       </c>
     </row>
     <row r="29" spans="1:18" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A29" s="153"/>
-      <c r="B29" s="152"/>
+      <c r="A29" s="150"/>
+      <c r="B29" s="137"/>
       <c r="C29" s="118" t="s">
         <v>36</v>
       </c>
@@ -2925,23 +2941,27 @@
         <v>36</v>
       </c>
       <c r="E29" s="50" t="s">
-        <v>47</v>
+        <v>76</v>
       </c>
       <c r="F29" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="G29" s="78"/>
+      <c r="G29" s="50" t="s">
+        <v>77</v>
+      </c>
       <c r="H29" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="I29" s="28"/>
+      <c r="I29" s="158" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="30" spans="1:18" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A30" s="154">
+      <c r="A30" s="151">
         <f>A28 -1</f>
         <v>4</v>
       </c>
-      <c r="B30" s="146" t="s">
+      <c r="B30" s="136" t="s">
         <v>13</v>
       </c>
       <c r="C30" s="59">
@@ -2974,14 +2994,14 @@
       </c>
     </row>
     <row r="31" spans="1:18" ht="93" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="143"/>
-      <c r="B31" s="147"/>
+      <c r="A31" s="142"/>
+      <c r="B31" s="138"/>
       <c r="C31" s="29"/>
       <c r="D31" s="106" t="s">
         <v>24</v>
       </c>
       <c r="E31" s="107" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F31" s="12" t="s">
         <v>42</v>
@@ -2993,11 +3013,11 @@
       <c r="I31" s="28"/>
     </row>
     <row r="32" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A32" s="143">
+      <c r="A32" s="142">
         <f>A30 -1</f>
         <v>3</v>
       </c>
-      <c r="B32" s="147"/>
+      <c r="B32" s="138"/>
       <c r="C32" s="27">
         <f>I30 + 1</f>
         <v>14</v>
@@ -3028,8 +3048,8 @@
       </c>
     </row>
     <row r="33" spans="1:9" ht="38.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" s="143"/>
-      <c r="B33" s="147"/>
+      <c r="A33" s="142"/>
+      <c r="B33" s="138"/>
       <c r="C33" s="29"/>
       <c r="D33" s="102" t="s">
         <v>6</v>
@@ -3045,11 +3065,11 @@
       <c r="I33" s="28"/>
     </row>
     <row r="34" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A34" s="143">
+      <c r="A34" s="142">
         <f>A32 -1</f>
         <v>2</v>
       </c>
-      <c r="B34" s="147"/>
+      <c r="B34" s="138"/>
       <c r="C34" s="29">
         <f>I32 + 1</f>
         <v>21</v>
@@ -3080,8 +3100,8 @@
       </c>
     </row>
     <row r="35" spans="1:9" ht="64.150000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A35" s="148"/>
-      <c r="B35" s="152"/>
+      <c r="A35" s="143"/>
+      <c r="B35" s="137"/>
       <c r="C35" s="57"/>
       <c r="D35" s="43" t="s">
         <v>21</v>
@@ -3097,11 +3117,11 @@
       <c r="I35" s="41"/>
     </row>
     <row r="36" spans="1:9" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A36" s="140">
+      <c r="A36" s="144">
         <f>A34 -1</f>
         <v>1</v>
       </c>
-      <c r="B36" s="149" t="s">
+      <c r="B36" s="139" t="s">
         <v>34</v>
       </c>
       <c r="C36" s="17">
@@ -3133,8 +3153,8 @@
       </c>
     </row>
     <row r="37" spans="1:9" ht="58.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A37" s="141"/>
-      <c r="B37" s="145"/>
+      <c r="A37" s="145"/>
+      <c r="B37" s="140"/>
       <c r="C37" s="96"/>
       <c r="D37" s="49" t="s">
         <v>6</v>
@@ -3152,10 +3172,10 @@
       </c>
     </row>
     <row r="38" spans="1:9" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A38" s="155" t="s">
+      <c r="A38" s="146" t="s">
         <v>25</v>
       </c>
-      <c r="B38" s="144" t="s">
+      <c r="B38" s="141" t="s">
         <v>5</v>
       </c>
       <c r="C38" s="20">
@@ -3188,8 +3208,8 @@
       </c>
     </row>
     <row r="39" spans="1:9" ht="134.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A39" s="156"/>
-      <c r="B39" s="145"/>
+      <c r="A39" s="147"/>
+      <c r="B39" s="140"/>
       <c r="C39" s="60" t="s">
         <v>39</v>
       </c>
@@ -3207,18 +3227,6 @@
     <row r="40" spans="1:9" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="B30:B35"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="A36:A37"/>
-    <mergeCell ref="A38:A39"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="A30:A31"/>
-    <mergeCell ref="A32:A33"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A22:A23"/>
     <mergeCell ref="A3:A4"/>
@@ -3235,6 +3243,18 @@
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="B13:B14"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="B30:B35"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="A38:A39"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0" footer="0"/>

</xml_diff>

<commit_message>
updated schedule, due dates, and calendar, removed exam
</commit_message>
<xml_diff>
--- a/CS320-Spring2024Calendar.xlsx
+++ b/CS320-Spring2024Calendar.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cygwin64\home\donha\cs320-spring2024\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A928314-B451-4BB0-A278-11C54AB98939}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{252AC9EE-1339-462D-ADB8-26A7FFBDE9DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="368" yWindow="368" windowWidth="19830" windowHeight="15127" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2205" yWindow="1073" windowWidth="23198" windowHeight="15127" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calendar-Sp24" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="82">
   <si>
     <t>Monday</t>
   </si>
@@ -182,12 +182,6 @@
     </r>
   </si>
   <si>
-    <t>A10: Team Project Reflection due
-A11: Team Project
-Final Self/Peer Evaluations due
-both due Noon (Marmoset)</t>
-  </si>
-  <si>
     <t>Lab 1: HTML &amp; CSS  Resume
 due Noon
 (Marmoset)</t>
@@ -196,24 +190,6 @@
     <t>Library Example Project
 Analysis and
 Review</t>
-  </si>
-  <si>
-    <t>FINAL EXAM PERIOD
-Section 101:
-10:15a to 12:15p
-A08: Team Presentation and Demonstration
-(in class)</t>
-  </si>
-  <si>
-    <t>FINAL EXAM PERIOD
-Section 102:
-12:45p to 2:45p
-A08: Team Presentation and Demonstration
-(in class)</t>
-  </si>
-  <si>
-    <t>A08: Team Report due Noon
-(Marmoset)</t>
   </si>
   <si>
     <t>A11: Team Project Midterm
@@ -557,43 +533,6 @@
     <t>ORM Review (Lab06)</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Team Session
-(in class)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Take Home Exam
-(due in class)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Work Ethic Lecture
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Take Home Exam
-(handed out)</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">
 A09: Individual  Report 
 due 4-10-24
@@ -609,7 +548,32 @@
   </si>
   <si>
     <t>CS320: SW Engineering - Spring 2024 Schedule
-(as of 4-12-2024, subject to change)</t>
+(as of 4-23-2024, subject to change)</t>
+  </si>
+  <si>
+    <t>Work Ethic
+Lecture</t>
+  </si>
+  <si>
+    <t>A08: Final Team Presentation and Demonstration
+FINAL EXAM PERIOD
+Section 101:
+10:15a to 12:15p</t>
+  </si>
+  <si>
+    <t>A08: Final Team Presentation and Demonstration
+FINAL EXAM PERIOD
+Section 102:
+12:45p to 2:45p</t>
+  </si>
+  <si>
+    <t>A10/A11: Team Project Self Reflection and 
+Final Peer Evals
+due Noon (Marmoset)</t>
+  </si>
+  <si>
+    <t>A08: Team Project Report due Noon
+(Marmoset)</t>
   </si>
 </sst>
 </file>
@@ -1311,7 +1275,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="158">
+  <cellXfs count="157">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1598,9 +1562,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1664,9 +1625,6 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1715,53 +1673,65 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
@@ -1769,20 +1739,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2111,17 +2072,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="53.1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="136" t="s">
-        <v>82</v>
-      </c>
-      <c r="B1" s="137"/>
-      <c r="C1" s="137"/>
-      <c r="D1" s="137"/>
-      <c r="E1" s="137"/>
-      <c r="F1" s="137"/>
-      <c r="G1" s="137"/>
-      <c r="H1" s="137"/>
-      <c r="I1" s="138"/>
+      <c r="A1" s="149" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" s="150"/>
+      <c r="C1" s="150"/>
+      <c r="D1" s="150"/>
+      <c r="E1" s="150"/>
+      <c r="F1" s="150"/>
+      <c r="G1" s="150"/>
+      <c r="H1" s="150"/>
+      <c r="I1" s="151"/>
     </row>
     <row r="2" spans="1:18" s="2" customFormat="1" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A2" s="1" t="s">
@@ -2154,7 +2115,7 @@
       <c r="A3" s="141">
         <v>15</v>
       </c>
-      <c r="B3" s="150" t="s">
+      <c r="B3" s="136" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="66">
@@ -2186,8 +2147,8 @@
       </c>
     </row>
     <row r="4" spans="1:18" ht="75.400000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A4" s="140"/>
-      <c r="B4" s="151"/>
+      <c r="A4" s="145"/>
+      <c r="B4" s="153"/>
       <c r="C4" s="68" t="s">
         <v>7</v>
       </c>
@@ -2208,16 +2169,16 @@
       </c>
       <c r="G4" s="37"/>
       <c r="H4" s="36" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I4" s="40"/>
     </row>
     <row r="5" spans="1:18" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="140">
+      <c r="A5" s="145">
         <f>A3 - 1</f>
         <v>14</v>
       </c>
-      <c r="B5" s="145" t="s">
+      <c r="B5" s="138" t="s">
         <v>27</v>
       </c>
       <c r="C5" s="7">
@@ -2250,29 +2211,29 @@
     </row>
     <row r="6" spans="1:18" ht="146.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A6" s="142"/>
-      <c r="B6" s="146"/>
-      <c r="C6" s="115" t="s">
-        <v>48</v>
-      </c>
-      <c r="D6" s="120" t="s">
-        <v>50</v>
+      <c r="B6" s="137"/>
+      <c r="C6" s="114" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="118" t="s">
+        <v>46</v>
       </c>
       <c r="E6" s="56"/>
-      <c r="F6" s="116" t="s">
-        <v>51</v>
+      <c r="F6" s="115" t="s">
+        <v>47</v>
       </c>
       <c r="G6" s="48"/>
       <c r="H6" s="47" t="s">
-        <v>53</v>
-      </c>
-      <c r="I6" s="103"/>
+        <v>49</v>
+      </c>
+      <c r="I6" s="102"/>
     </row>
     <row r="7" spans="1:18" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="143">
+      <c r="A7" s="146">
         <f>A5 - 1</f>
         <v>13</v>
       </c>
-      <c r="B7" s="147" t="s">
+      <c r="B7" s="133" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="38">
@@ -2305,30 +2266,30 @@
       </c>
     </row>
     <row r="8" spans="1:18" ht="99.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="144"/>
-      <c r="B8" s="148"/>
+      <c r="A8" s="139"/>
+      <c r="B8" s="135"/>
       <c r="C8" s="30" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D8" s="47" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E8" s="10"/>
       <c r="F8" s="12" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="G8" s="27"/>
       <c r="H8" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="I8" s="125"/>
+        <v>54</v>
+      </c>
+      <c r="I8" s="123"/>
     </row>
     <row r="9" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="144">
+      <c r="A9" s="139">
         <f>A7 - 1</f>
         <v>12</v>
       </c>
-      <c r="B9" s="148"/>
+      <c r="B9" s="135"/>
       <c r="C9" s="14">
         <f>I7 + 1</f>
         <v>11</v>
@@ -2357,48 +2318,48 @@
         <f t="shared" si="1"/>
         <v>17</v>
       </c>
-      <c r="L9" s="109"/>
-      <c r="M9" s="109"/>
-      <c r="N9" s="109"/>
-      <c r="O9" s="109"/>
-      <c r="P9" s="109"/>
-      <c r="Q9" s="109"/>
-      <c r="R9" s="109"/>
+      <c r="L9" s="108"/>
+      <c r="M9" s="108"/>
+      <c r="N9" s="108"/>
+      <c r="O9" s="108"/>
+      <c r="P9" s="108"/>
+      <c r="Q9" s="108"/>
+      <c r="R9" s="108"/>
     </row>
     <row r="10" spans="1:18" ht="102.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="144"/>
-      <c r="B10" s="148"/>
-      <c r="C10" s="124" t="s">
+      <c r="A10" s="139"/>
+      <c r="B10" s="135"/>
+      <c r="C10" s="122" t="s">
         <v>37</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="E10" s="104" t="s">
-        <v>59</v>
+      <c r="E10" s="103" t="s">
+        <v>55</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="G10" s="11"/>
       <c r="H10" s="10" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="I10" s="13"/>
       <c r="L10" s="25"/>
-      <c r="M10" s="109"/>
-      <c r="N10" s="110"/>
-      <c r="O10" s="109"/>
-      <c r="P10" s="110"/>
-      <c r="Q10" s="109"/>
-      <c r="R10" s="110"/>
+      <c r="M10" s="108"/>
+      <c r="N10" s="109"/>
+      <c r="O10" s="108"/>
+      <c r="P10" s="109"/>
+      <c r="Q10" s="108"/>
+      <c r="R10" s="109"/>
     </row>
     <row r="11" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="144">
+      <c r="A11" s="139">
         <f>A9 -1</f>
         <v>11</v>
       </c>
-      <c r="B11" s="148"/>
+      <c r="B11" s="135"/>
       <c r="C11" s="17">
         <f>I9 + 1</f>
         <v>18</v>
@@ -2427,48 +2388,48 @@
         <f t="shared" si="1"/>
         <v>24</v>
       </c>
-      <c r="L11" s="109"/>
-      <c r="M11" s="109"/>
-      <c r="N11" s="109"/>
-      <c r="O11" s="109"/>
-      <c r="P11" s="109"/>
-      <c r="Q11" s="109"/>
-      <c r="R11" s="109"/>
+      <c r="L11" s="108"/>
+      <c r="M11" s="108"/>
+      <c r="N11" s="108"/>
+      <c r="O11" s="108"/>
+      <c r="P11" s="108"/>
+      <c r="Q11" s="108"/>
+      <c r="R11" s="108"/>
     </row>
     <row r="12" spans="1:18" ht="115.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A12" s="144"/>
-      <c r="B12" s="148"/>
+      <c r="A12" s="139"/>
+      <c r="B12" s="135"/>
       <c r="C12" s="30" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D12" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="E12" s="131" t="s">
-        <v>62</v>
+      <c r="E12" s="129" t="s">
+        <v>58</v>
       </c>
       <c r="F12" s="44" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="G12" s="42"/>
-      <c r="H12" s="127" t="s">
-        <v>64</v>
+      <c r="H12" s="125" t="s">
+        <v>60</v>
       </c>
       <c r="I12" s="77"/>
       <c r="L12" s="25"/>
-      <c r="M12" s="109"/>
-      <c r="N12" s="109"/>
-      <c r="O12" s="109"/>
-      <c r="P12" s="110"/>
-      <c r="Q12" s="109"/>
-      <c r="R12" s="110"/>
+      <c r="M12" s="108"/>
+      <c r="N12" s="108"/>
+      <c r="O12" s="108"/>
+      <c r="P12" s="109"/>
+      <c r="Q12" s="108"/>
+      <c r="R12" s="109"/>
     </row>
     <row r="13" spans="1:18" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="144">
+      <c r="A13" s="139">
         <f xml:space="preserve"> A11 - 1</f>
         <v>10</v>
       </c>
-      <c r="B13" s="152" t="s">
+      <c r="B13" s="154" t="s">
         <v>28</v>
       </c>
       <c r="C13" s="17">
@@ -2498,25 +2459,25 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L13" s="109"/>
-      <c r="M13" s="109"/>
-      <c r="N13" s="109"/>
-      <c r="O13" s="109"/>
-      <c r="P13" s="109"/>
-      <c r="Q13" s="109"/>
-      <c r="R13" s="111"/>
+      <c r="L13" s="108"/>
+      <c r="M13" s="108"/>
+      <c r="N13" s="108"/>
+      <c r="O13" s="108"/>
+      <c r="P13" s="108"/>
+      <c r="Q13" s="108"/>
+      <c r="R13" s="110"/>
     </row>
     <row r="14" spans="1:18" ht="100.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A14" s="149"/>
-      <c r="B14" s="153"/>
-      <c r="C14" s="128" t="s">
-        <v>60</v>
-      </c>
-      <c r="D14" s="122" t="s">
-        <v>66</v>
+      <c r="A14" s="140"/>
+      <c r="B14" s="134"/>
+      <c r="C14" s="126" t="s">
+        <v>56</v>
+      </c>
+      <c r="D14" s="120" t="s">
+        <v>62</v>
       </c>
       <c r="E14" s="89"/>
-      <c r="F14" s="121" t="s">
+      <c r="F14" s="119" t="s">
         <v>22</v>
       </c>
       <c r="G14" s="88" t="s">
@@ -2528,20 +2489,20 @@
       <c r="I14" s="84" t="s">
         <v>32</v>
       </c>
-      <c r="L14" s="111"/>
+      <c r="L14" s="110"/>
       <c r="M14" s="25"/>
-      <c r="N14" s="112"/>
-      <c r="O14" s="109"/>
-      <c r="P14" s="111"/>
-      <c r="Q14" s="109"/>
-      <c r="R14" s="111"/>
+      <c r="N14" s="111"/>
+      <c r="O14" s="108"/>
+      <c r="P14" s="110"/>
+      <c r="Q14" s="108"/>
+      <c r="R14" s="110"/>
     </row>
     <row r="15" spans="1:18" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
       <c r="A15" s="141">
         <f>A13 - 1</f>
         <v>9</v>
       </c>
-      <c r="B15" s="145" t="s">
+      <c r="B15" s="138" t="s">
         <v>12</v>
       </c>
       <c r="C15" s="66">
@@ -2575,12 +2536,12 @@
     </row>
     <row r="16" spans="1:18" ht="103.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A16" s="142"/>
-      <c r="B16" s="146"/>
+      <c r="B16" s="137"/>
       <c r="C16" s="85" t="s">
         <v>32</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E16" s="63" t="s">
         <v>26</v>
@@ -2602,8 +2563,8 @@
 Team MS1 Prep
 (all in-class)</v>
       </c>
-      <c r="I16" s="132" t="s">
-        <v>61</v>
+      <c r="I16" s="130" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:18" ht="6.4" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
@@ -2625,13 +2586,13 @@
         <v>15</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="F18" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="G18" s="119" t="s">
-        <v>47</v>
+      <c r="G18" s="117" t="s">
+        <v>43</v>
       </c>
       <c r="H18" s="33" t="s">
         <v>17</v>
@@ -2640,31 +2601,31 @@
         <v>29</v>
       </c>
     </row>
-    <row r="19" spans="1:18" s="114" customFormat="1" ht="21.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A19" s="113"/>
+    <row r="19" spans="1:18" s="113" customFormat="1" ht="21.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A19" s="112"/>
       <c r="B19" s="34"/>
       <c r="C19" s="34"/>
-      <c r="D19" s="111"/>
-      <c r="E19" s="111"/>
-      <c r="F19" s="111"/>
-      <c r="G19" s="111"/>
-      <c r="H19" s="111"/>
-      <c r="I19" s="111"/>
+      <c r="D19" s="110"/>
+      <c r="E19" s="110"/>
+      <c r="F19" s="110"/>
+      <c r="G19" s="110"/>
+      <c r="H19" s="110"/>
+      <c r="I19" s="110"/>
     </row>
     <row r="20" spans="1:18" ht="54" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A20" s="136" t="str">
+      <c r="A20" s="149" t="str">
         <f>A1</f>
         <v>CS320: SW Engineering - Spring 2024 Schedule
-(as of 4-12-2024, subject to change)</v>
-      </c>
-      <c r="B20" s="137"/>
-      <c r="C20" s="137"/>
-      <c r="D20" s="137"/>
-      <c r="E20" s="137"/>
-      <c r="F20" s="137"/>
-      <c r="G20" s="137"/>
-      <c r="H20" s="137"/>
-      <c r="I20" s="138"/>
+(as of 4-23-2024, subject to change)</v>
+      </c>
+      <c r="B20" s="150"/>
+      <c r="C20" s="150"/>
+      <c r="D20" s="150"/>
+      <c r="E20" s="150"/>
+      <c r="F20" s="150"/>
+      <c r="G20" s="150"/>
+      <c r="H20" s="150"/>
+      <c r="I20" s="151"/>
     </row>
     <row r="21" spans="1:18" s="2" customFormat="1" ht="17.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A21" s="1" t="str">
@@ -2702,11 +2663,11 @@
       </c>
     </row>
     <row r="22" spans="1:18" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="139">
+      <c r="A22" s="152">
         <f>A15-1</f>
         <v>8</v>
       </c>
-      <c r="B22" s="145" t="s">
+      <c r="B22" s="138" t="s">
         <v>12</v>
       </c>
       <c r="C22" s="93">
@@ -2737,44 +2698,44 @@
         <f t="shared" si="5"/>
         <v>16</v>
       </c>
-      <c r="L22" s="111"/>
-      <c r="M22" s="109"/>
-      <c r="N22" s="109"/>
-      <c r="O22" s="109"/>
-      <c r="P22" s="109"/>
-      <c r="Q22" s="109"/>
-      <c r="R22" s="109"/>
+      <c r="L22" s="110"/>
+      <c r="M22" s="108"/>
+      <c r="N22" s="108"/>
+      <c r="O22" s="108"/>
+      <c r="P22" s="108"/>
+      <c r="Q22" s="108"/>
+      <c r="R22" s="108"/>
     </row>
     <row r="23" spans="1:18" ht="67.150000000000006" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A23" s="140"/>
-      <c r="B23" s="145"/>
-      <c r="C23" s="133"/>
+      <c r="A23" s="145"/>
+      <c r="B23" s="138"/>
+      <c r="C23" s="131"/>
       <c r="D23" s="6" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E23" s="54"/>
       <c r="F23" s="6" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G23" s="6"/>
       <c r="H23" s="22" t="s">
         <v>14</v>
       </c>
       <c r="I23" s="35"/>
-      <c r="L23" s="109"/>
-      <c r="M23" s="109"/>
-      <c r="N23" s="109"/>
-      <c r="O23" s="109"/>
-      <c r="P23" s="109"/>
-      <c r="Q23" s="109"/>
+      <c r="L23" s="108"/>
+      <c r="M23" s="108"/>
+      <c r="N23" s="108"/>
+      <c r="O23" s="108"/>
+      <c r="P23" s="108"/>
+      <c r="Q23" s="108"/>
       <c r="R23" s="25"/>
     </row>
     <row r="24" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A24" s="140">
+      <c r="A24" s="145">
         <f>A22 - 1</f>
         <v>7</v>
       </c>
-      <c r="B24" s="145"/>
+      <c r="B24" s="138"/>
       <c r="C24" s="7">
         <f>I22 + 1</f>
         <v>17</v>
@@ -2803,44 +2764,44 @@
         <f t="shared" si="6"/>
         <v>23</v>
       </c>
-      <c r="L24" s="109"/>
-      <c r="M24" s="109"/>
-      <c r="N24" s="109"/>
-      <c r="O24" s="109"/>
-      <c r="P24" s="109"/>
-      <c r="Q24" s="109"/>
-      <c r="R24" s="109"/>
+      <c r="L24" s="108"/>
+      <c r="M24" s="108"/>
+      <c r="N24" s="108"/>
+      <c r="O24" s="108"/>
+      <c r="P24" s="108"/>
+      <c r="Q24" s="108"/>
+      <c r="R24" s="108"/>
     </row>
     <row r="25" spans="1:18" ht="124.15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="140"/>
-      <c r="B25" s="145"/>
-      <c r="C25" s="108"/>
+      <c r="A25" s="145"/>
+      <c r="B25" s="138"/>
+      <c r="C25" s="107"/>
       <c r="D25" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="E25" s="126"/>
+      <c r="E25" s="124"/>
       <c r="F25" s="54" t="s">
         <v>38</v>
       </c>
-      <c r="G25" s="126"/>
-      <c r="H25" s="134" t="s">
-        <v>69</v>
-      </c>
-      <c r="I25" s="130"/>
+      <c r="G25" s="124"/>
+      <c r="H25" s="132" t="s">
+        <v>65</v>
+      </c>
+      <c r="I25" s="128"/>
       <c r="L25" s="25"/>
-      <c r="M25" s="109"/>
-      <c r="N25" s="111"/>
-      <c r="O25" s="109"/>
-      <c r="P25" s="111"/>
-      <c r="Q25" s="109"/>
+      <c r="M25" s="108"/>
+      <c r="N25" s="110"/>
+      <c r="O25" s="108"/>
+      <c r="P25" s="110"/>
+      <c r="Q25" s="108"/>
       <c r="R25" s="25"/>
     </row>
     <row r="26" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A26" s="140">
+      <c r="A26" s="145">
         <f>A24 - 1</f>
         <v>6</v>
       </c>
-      <c r="B26" s="145"/>
+      <c r="B26" s="138"/>
       <c r="C26" s="7">
         <f>I24 + 1</f>
         <v>24</v>
@@ -2861,7 +2822,7 @@
         <f t="shared" si="7"/>
         <v>28</v>
       </c>
-      <c r="H26" s="98">
+      <c r="H26" s="97">
         <f t="shared" ref="H26" si="8">G26 + 1</f>
         <v>29</v>
       </c>
@@ -2869,57 +2830,57 @@
         <f t="shared" ref="I26" si="9">H26 + 1</f>
         <v>30</v>
       </c>
-      <c r="L26" s="109"/>
-      <c r="M26" s="109"/>
-      <c r="N26" s="109"/>
-      <c r="O26" s="109"/>
-      <c r="P26" s="109"/>
-      <c r="Q26" s="109"/>
-      <c r="R26" s="109"/>
+      <c r="L26" s="108"/>
+      <c r="M26" s="108"/>
+      <c r="N26" s="108"/>
+      <c r="O26" s="108"/>
+      <c r="P26" s="108"/>
+      <c r="Q26" s="108"/>
+      <c r="R26" s="108"/>
     </row>
     <row r="27" spans="1:18" ht="68.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A27" s="142"/>
-      <c r="B27" s="146"/>
-      <c r="C27" s="129" t="s">
-        <v>70</v>
+      <c r="B27" s="137"/>
+      <c r="C27" s="127" t="s">
+        <v>66</v>
       </c>
       <c r="D27" s="9" t="s">
         <v>20</v>
       </c>
       <c r="E27" s="54"/>
       <c r="F27" s="23" t="s">
-        <v>71</v>
-      </c>
-      <c r="G27" s="123" t="s">
-        <v>45</v>
+        <v>67</v>
+      </c>
+      <c r="G27" s="121" t="s">
+        <v>41</v>
       </c>
       <c r="H27" s="71" t="s">
         <v>36</v>
       </c>
-      <c r="I27" s="107" t="s">
+      <c r="I27" s="106" t="s">
         <v>36</v>
       </c>
-      <c r="L27" s="109"/>
-      <c r="M27" s="109"/>
+      <c r="L27" s="108"/>
+      <c r="M27" s="108"/>
       <c r="N27" s="25"/>
-      <c r="O27" s="109"/>
+      <c r="O27" s="108"/>
       <c r="P27" s="25"/>
-      <c r="Q27" s="111"/>
+      <c r="Q27" s="110"/>
       <c r="R27" s="25"/>
     </row>
     <row r="28" spans="1:18" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A28" s="143">
+      <c r="A28" s="146">
         <f>A26 -1</f>
         <v>5</v>
       </c>
-      <c r="B28" s="147" t="s">
+      <c r="B28" s="133" t="s">
         <v>33</v>
       </c>
-      <c r="C28" s="99">
+      <c r="C28" s="98">
         <f>I26 + 1</f>
         <v>31</v>
       </c>
-      <c r="D28" s="100">
+      <c r="D28" s="99">
         <v>1</v>
       </c>
       <c r="E28" s="39">
@@ -2944,34 +2905,34 @@
       </c>
     </row>
     <row r="29" spans="1:18" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A29" s="154"/>
-      <c r="B29" s="153"/>
-      <c r="C29" s="117" t="s">
+      <c r="A29" s="147"/>
+      <c r="B29" s="134"/>
+      <c r="C29" s="116" t="s">
         <v>36</v>
       </c>
-      <c r="D29" s="101" t="s">
+      <c r="D29" s="100" t="s">
         <v>36</v>
       </c>
       <c r="E29" s="50" t="s">
+        <v>68</v>
+      </c>
+      <c r="F29" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="G29" s="50" t="s">
+        <v>69</v>
+      </c>
+      <c r="H29" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="F29" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="G29" s="50" t="s">
-        <v>73</v>
-      </c>
-      <c r="H29" s="12" t="s">
-        <v>76</v>
-      </c>
       <c r="I29" s="28"/>
     </row>
     <row r="30" spans="1:18" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A30" s="155">
+      <c r="A30" s="148">
         <f>A28 -1</f>
         <v>4</v>
       </c>
-      <c r="B30" s="147" t="s">
+      <c r="B30" s="133" t="s">
         <v>13</v>
       </c>
       <c r="C30" s="59">
@@ -3004,32 +2965,32 @@
       </c>
     </row>
     <row r="31" spans="1:18" ht="87.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="144"/>
-      <c r="B31" s="148"/>
+      <c r="A31" s="139"/>
+      <c r="B31" s="135"/>
       <c r="C31" s="30" t="s">
+        <v>70</v>
+      </c>
+      <c r="D31" s="104" t="s">
+        <v>24</v>
+      </c>
+      <c r="E31" s="105" t="s">
         <v>74</v>
       </c>
-      <c r="D31" s="105" t="s">
-        <v>24</v>
-      </c>
-      <c r="E31" s="106" t="s">
-        <v>80</v>
-      </c>
       <c r="F31" s="12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G31" s="27"/>
       <c r="H31" s="27" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="I31" s="28"/>
     </row>
     <row r="32" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A32" s="144">
+      <c r="A32" s="139">
         <f>A30 -1</f>
         <v>3</v>
       </c>
-      <c r="B32" s="148"/>
+      <c r="B32" s="135"/>
       <c r="C32" s="27">
         <f>I30 + 1</f>
         <v>14</v>
@@ -3060,15 +3021,15 @@
       </c>
     </row>
     <row r="33" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" s="144"/>
-      <c r="B33" s="148"/>
+      <c r="A33" s="139"/>
+      <c r="B33" s="135"/>
       <c r="C33" s="29"/>
-      <c r="D33" s="102" t="s">
+      <c r="D33" s="101" t="s">
         <v>6</v>
       </c>
       <c r="E33" s="11"/>
       <c r="F33" s="44" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="G33" s="78"/>
       <c r="H33" s="12" t="s">
@@ -3077,11 +3038,11 @@
       <c r="I33" s="28"/>
     </row>
     <row r="34" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A34" s="144">
+      <c r="A34" s="139">
         <f>A32 -1</f>
         <v>2</v>
       </c>
-      <c r="B34" s="148"/>
+      <c r="B34" s="135"/>
       <c r="C34" s="29">
         <f>I32 + 1</f>
         <v>21</v>
@@ -3111,20 +3072,20 @@
         <v>27</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="63.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A35" s="149"/>
-      <c r="B35" s="153"/>
+    <row r="35" spans="1:9" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A35" s="140"/>
+      <c r="B35" s="134"/>
       <c r="C35" s="57"/>
       <c r="D35" s="43" t="s">
         <v>21</v>
       </c>
       <c r="E35" s="42"/>
       <c r="F35" s="44" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G35" s="42"/>
-      <c r="H35" s="135" t="s">
-        <v>78</v>
+      <c r="H35" s="155" t="s">
+        <v>6</v>
       </c>
       <c r="I35" s="41"/>
     </row>
@@ -3133,7 +3094,7 @@
         <f>A34 -1</f>
         <v>1</v>
       </c>
-      <c r="B36" s="150" t="s">
+      <c r="B36" s="136" t="s">
         <v>34</v>
       </c>
       <c r="C36" s="17">
@@ -3164,14 +3125,16 @@
         <v>4</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="53.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="37" spans="1:9" ht="85.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A37" s="142"/>
-      <c r="B37" s="146"/>
-      <c r="C37" s="96"/>
+      <c r="B37" s="137"/>
+      <c r="C37" s="60" t="s">
+        <v>80</v>
+      </c>
       <c r="D37" s="49" t="s">
         <v>6</v>
       </c>
-      <c r="E37" s="97"/>
+      <c r="E37" s="96"/>
       <c r="F37" s="95" t="s">
         <v>6</v>
       </c>
@@ -3179,15 +3142,13 @@
       <c r="H37" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="I37" s="118" t="s">
-        <v>44</v>
-      </c>
+      <c r="I37" s="91"/>
     </row>
     <row r="38" spans="1:9" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A38" s="156" t="s">
+      <c r="A38" s="143" t="s">
         <v>25</v>
       </c>
-      <c r="B38" s="145" t="s">
+      <c r="B38" s="138" t="s">
         <v>5</v>
       </c>
       <c r="C38" s="20">
@@ -3219,18 +3180,18 @@
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="134.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A39" s="157"/>
-      <c r="B39" s="146"/>
-      <c r="C39" s="60" t="s">
-        <v>39</v>
+    <row r="39" spans="1:9" ht="103.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A39" s="144"/>
+      <c r="B39" s="137"/>
+      <c r="C39" s="156" t="s">
+        <v>81</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>42</v>
+        <v>78</v>
       </c>
       <c r="E39" s="61"/>
       <c r="F39" s="23" t="s">
-        <v>43</v>
+        <v>79</v>
       </c>
       <c r="G39" s="21"/>
       <c r="H39" s="75"/>
@@ -3239,18 +3200,6 @@
     <row r="40" spans="1:9" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="B30:B35"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="A36:A37"/>
-    <mergeCell ref="A38:A39"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="A30:A31"/>
-    <mergeCell ref="A32:A33"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A22:A23"/>
     <mergeCell ref="A3:A4"/>
@@ -3267,6 +3216,18 @@
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="B13:B14"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="B30:B35"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="A38:A39"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0" footer="0"/>

</xml_diff>

<commit_message>
updated calendar and added bolwing data to resources
</commit_message>
<xml_diff>
--- a/CS320-Spring2024Calendar.xlsx
+++ b/CS320-Spring2024Calendar.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cygwin64\home\donha\cs320-spring2024\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{252AC9EE-1339-462D-ADB8-26A7FFBDE9DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{354855EC-2D25-4230-BA43-64A7AEEDA5DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2205" yWindow="1073" windowWidth="23198" windowHeight="15127" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="165" windowWidth="22815" windowHeight="15128" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calendar-Sp24" sheetId="1" r:id="rId1"/>
@@ -541,16 +541,6 @@
 (Marmoset)</t>
   </si>
   <si>
-    <t>SPARTAN DAY
-(class optional)
-Team Session
-(in class)</t>
-  </si>
-  <si>
-    <t>CS320: SW Engineering - Spring 2024 Schedule
-(as of 4-23-2024, subject to change)</t>
-  </si>
-  <si>
     <t>Work Ethic
 Lecture</t>
   </si>
@@ -572,8 +562,19 @@
 due Noon (Marmoset)</t>
   </si>
   <si>
-    <t>A08: Team Project Report due Noon
+    <t>CS320: SW Engineering - Spring 2024 Schedule
+(as of 5-5-2024, subject to change)</t>
+  </si>
+  <si>
+    <t>A08: Team Project Report
+ due Noon
 (Marmoset)</t>
+  </si>
+  <si>
+    <t>SPARTAN DAY
+(class optional)
+Creating a Database
+from CSV files</t>
   </si>
 </sst>
 </file>
@@ -1275,7 +1276,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="157">
+  <cellXfs count="155">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1337,9 +1338,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1672,35 +1670,65 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1709,40 +1737,7 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2072,17 +2067,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="53.1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="149" t="s">
-        <v>76</v>
-      </c>
-      <c r="B1" s="150"/>
-      <c r="C1" s="150"/>
-      <c r="D1" s="150"/>
-      <c r="E1" s="150"/>
-      <c r="F1" s="150"/>
-      <c r="G1" s="150"/>
-      <c r="H1" s="150"/>
-      <c r="I1" s="151"/>
+      <c r="A1" s="132" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1" s="133"/>
+      <c r="C1" s="133"/>
+      <c r="D1" s="133"/>
+      <c r="E1" s="133"/>
+      <c r="F1" s="133"/>
+      <c r="G1" s="133"/>
+      <c r="H1" s="133"/>
+      <c r="I1" s="134"/>
     </row>
     <row r="2" spans="1:18" s="2" customFormat="1" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A2" s="1" t="s">
@@ -2112,24 +2107,24 @@
       </c>
     </row>
     <row r="3" spans="1:18" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="141">
+      <c r="A3" s="137">
         <v>15</v>
       </c>
-      <c r="B3" s="136" t="s">
+      <c r="B3" s="146" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="66">
+      <c r="C3" s="65">
         <v>21</v>
       </c>
-      <c r="D3" s="64">
+      <c r="D3" s="63">
         <f>C3 + 1</f>
         <v>22</v>
       </c>
-      <c r="E3" s="64">
+      <c r="E3" s="63">
         <f t="shared" ref="E3:I3" si="0">D3 + 1</f>
         <v>23</v>
       </c>
-      <c r="F3" s="67">
+      <c r="F3" s="66">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
@@ -2147,38 +2142,38 @@
       </c>
     </row>
     <row r="4" spans="1:18" ht="75.400000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A4" s="145"/>
-      <c r="B4" s="153"/>
-      <c r="C4" s="68" t="s">
+      <c r="A4" s="136"/>
+      <c r="B4" s="147"/>
+      <c r="C4" s="67" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="65" t="str">
+      <c r="D4" s="64" t="str">
         <f xml:space="preserve"> C4</f>
         <v>SEMESTER
 BREAK</v>
       </c>
-      <c r="E4" s="69" t="str">
+      <c r="E4" s="68" t="str">
         <f>D4</f>
         <v>SEMESTER
 BREAK</v>
       </c>
-      <c r="F4" s="70" t="str">
+      <c r="F4" s="69" t="str">
         <f>E4</f>
         <v>SEMESTER
 BREAK</v>
       </c>
-      <c r="G4" s="37"/>
-      <c r="H4" s="36" t="s">
+      <c r="G4" s="36"/>
+      <c r="H4" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="I4" s="40"/>
+      <c r="I4" s="39"/>
     </row>
     <row r="5" spans="1:18" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="145">
+      <c r="A5" s="136">
         <f>A3 - 1</f>
         <v>14</v>
       </c>
-      <c r="B5" s="138" t="s">
+      <c r="B5" s="141" t="s">
         <v>27</v>
       </c>
       <c r="C5" s="7">
@@ -2197,50 +2192,50 @@
         <f t="shared" ref="E5:I13" si="1">E5 + 1</f>
         <v>31</v>
       </c>
-      <c r="G5" s="79">
+      <c r="G5" s="78">
         <v>1</v>
       </c>
-      <c r="H5" s="39">
+      <c r="H5" s="38">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="I5" s="46">
+      <c r="I5" s="45">
         <f>H5 + 1</f>
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:18" ht="146.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A6" s="142"/>
-      <c r="B6" s="137"/>
-      <c r="C6" s="114" t="s">
+      <c r="A6" s="138"/>
+      <c r="B6" s="142"/>
+      <c r="C6" s="113" t="s">
         <v>44</v>
       </c>
-      <c r="D6" s="118" t="s">
+      <c r="D6" s="117" t="s">
         <v>46</v>
       </c>
-      <c r="E6" s="56"/>
-      <c r="F6" s="115" t="s">
+      <c r="E6" s="55"/>
+      <c r="F6" s="114" t="s">
         <v>47</v>
       </c>
-      <c r="G6" s="48"/>
-      <c r="H6" s="47" t="s">
+      <c r="G6" s="47"/>
+      <c r="H6" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="I6" s="102"/>
+      <c r="I6" s="101"/>
     </row>
     <row r="7" spans="1:18" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="146">
+      <c r="A7" s="139">
         <f>A5 - 1</f>
         <v>13</v>
       </c>
-      <c r="B7" s="133" t="s">
+      <c r="B7" s="143" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="38">
+      <c r="C7" s="37">
         <f>I5 + 1</f>
         <v>4</v>
       </c>
-      <c r="D7" s="39">
+      <c r="D7" s="38">
         <f>C7 + 1</f>
         <v>5</v>
       </c>
@@ -2248,11 +2243,11 @@
         <f>D7 + 1</f>
         <v>6</v>
       </c>
-      <c r="F7" s="52">
+      <c r="F7" s="51">
         <f>E7+1</f>
         <v>7</v>
       </c>
-      <c r="G7" s="52">
+      <c r="G7" s="51">
         <f>F7+1</f>
         <v>8</v>
       </c>
@@ -2260,36 +2255,36 @@
         <f>G7 + 1</f>
         <v>9</v>
       </c>
-      <c r="I7" s="51">
+      <c r="I7" s="50">
         <f>H7+1</f>
         <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="99.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="139"/>
-      <c r="B8" s="135"/>
-      <c r="C8" s="30" t="s">
+      <c r="A8" s="140"/>
+      <c r="B8" s="144"/>
+      <c r="C8" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="47" t="s">
+      <c r="D8" s="46" t="s">
         <v>50</v>
       </c>
       <c r="E8" s="10"/>
       <c r="F8" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="G8" s="27"/>
+      <c r="G8" s="26"/>
       <c r="H8" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="I8" s="123"/>
+      <c r="I8" s="122"/>
     </row>
     <row r="9" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="139">
+      <c r="A9" s="140">
         <f>A7 - 1</f>
         <v>12</v>
       </c>
-      <c r="B9" s="135"/>
+      <c r="B9" s="144"/>
       <c r="C9" s="14">
         <f>I7 + 1</f>
         <v>11</v>
@@ -2318,24 +2313,24 @@
         <f t="shared" si="1"/>
         <v>17</v>
       </c>
-      <c r="L9" s="108"/>
-      <c r="M9" s="108"/>
-      <c r="N9" s="108"/>
-      <c r="O9" s="108"/>
-      <c r="P9" s="108"/>
-      <c r="Q9" s="108"/>
-      <c r="R9" s="108"/>
+      <c r="L9" s="107"/>
+      <c r="M9" s="107"/>
+      <c r="N9" s="107"/>
+      <c r="O9" s="107"/>
+      <c r="P9" s="107"/>
+      <c r="Q9" s="107"/>
+      <c r="R9" s="107"/>
     </row>
     <row r="10" spans="1:18" ht="102.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="139"/>
-      <c r="B10" s="135"/>
-      <c r="C10" s="122" t="s">
+      <c r="A10" s="140"/>
+      <c r="B10" s="144"/>
+      <c r="C10" s="121" t="s">
         <v>37</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="E10" s="103" t="s">
+      <c r="E10" s="102" t="s">
         <v>55</v>
       </c>
       <c r="F10" s="10" t="s">
@@ -2346,20 +2341,20 @@
         <v>52</v>
       </c>
       <c r="I10" s="13"/>
-      <c r="L10" s="25"/>
-      <c r="M10" s="108"/>
-      <c r="N10" s="109"/>
-      <c r="O10" s="108"/>
-      <c r="P10" s="109"/>
-      <c r="Q10" s="108"/>
-      <c r="R10" s="109"/>
+      <c r="L10" s="24"/>
+      <c r="M10" s="107"/>
+      <c r="N10" s="108"/>
+      <c r="O10" s="107"/>
+      <c r="P10" s="108"/>
+      <c r="Q10" s="107"/>
+      <c r="R10" s="108"/>
     </row>
     <row r="11" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="139">
+      <c r="A11" s="140">
         <f>A9 -1</f>
         <v>11</v>
       </c>
-      <c r="B11" s="135"/>
+      <c r="B11" s="144"/>
       <c r="C11" s="17">
         <f>I9 + 1</f>
         <v>18</v>
@@ -2388,55 +2383,55 @@
         <f t="shared" si="1"/>
         <v>24</v>
       </c>
-      <c r="L11" s="108"/>
-      <c r="M11" s="108"/>
-      <c r="N11" s="108"/>
-      <c r="O11" s="108"/>
-      <c r="P11" s="108"/>
-      <c r="Q11" s="108"/>
-      <c r="R11" s="108"/>
+      <c r="L11" s="107"/>
+      <c r="M11" s="107"/>
+      <c r="N11" s="107"/>
+      <c r="O11" s="107"/>
+      <c r="P11" s="107"/>
+      <c r="Q11" s="107"/>
+      <c r="R11" s="107"/>
     </row>
     <row r="12" spans="1:18" ht="115.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A12" s="139"/>
-      <c r="B12" s="135"/>
-      <c r="C12" s="30" t="s">
+      <c r="A12" s="140"/>
+      <c r="B12" s="144"/>
+      <c r="C12" s="29" t="s">
         <v>59</v>
       </c>
       <c r="D12" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="E12" s="129" t="s">
+      <c r="E12" s="128" t="s">
         <v>58</v>
       </c>
-      <c r="F12" s="44" t="s">
+      <c r="F12" s="43" t="s">
         <v>61</v>
       </c>
-      <c r="G12" s="42"/>
-      <c r="H12" s="125" t="s">
+      <c r="G12" s="41"/>
+      <c r="H12" s="124" t="s">
         <v>60</v>
       </c>
-      <c r="I12" s="77"/>
-      <c r="L12" s="25"/>
-      <c r="M12" s="108"/>
-      <c r="N12" s="108"/>
-      <c r="O12" s="108"/>
-      <c r="P12" s="109"/>
-      <c r="Q12" s="108"/>
-      <c r="R12" s="109"/>
+      <c r="I12" s="76"/>
+      <c r="L12" s="24"/>
+      <c r="M12" s="107"/>
+      <c r="N12" s="107"/>
+      <c r="O12" s="107"/>
+      <c r="P12" s="108"/>
+      <c r="Q12" s="107"/>
+      <c r="R12" s="108"/>
     </row>
     <row r="13" spans="1:18" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="139">
+      <c r="A13" s="140">
         <f xml:space="preserve"> A11 - 1</f>
         <v>10</v>
       </c>
-      <c r="B13" s="154" t="s">
+      <c r="B13" s="148" t="s">
         <v>28</v>
       </c>
       <c r="C13" s="17">
         <f>I11 + 1</f>
         <v>25</v>
       </c>
-      <c r="D13" s="81">
+      <c r="D13" s="80">
         <f>C13 + 1</f>
         <v>26</v>
       </c>
@@ -2448,102 +2443,102 @@
         <f t="shared" si="2"/>
         <v>28</v>
       </c>
-      <c r="G13" s="86">
+      <c r="G13" s="85">
         <f t="shared" si="2"/>
         <v>29</v>
       </c>
-      <c r="H13" s="73">
+      <c r="H13" s="72">
         <v>1</v>
       </c>
-      <c r="I13" s="87">
+      <c r="I13" s="86">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L13" s="108"/>
-      <c r="M13" s="108"/>
-      <c r="N13" s="108"/>
-      <c r="O13" s="108"/>
-      <c r="P13" s="108"/>
-      <c r="Q13" s="108"/>
-      <c r="R13" s="110"/>
+      <c r="L13" s="107"/>
+      <c r="M13" s="107"/>
+      <c r="N13" s="107"/>
+      <c r="O13" s="107"/>
+      <c r="P13" s="107"/>
+      <c r="Q13" s="107"/>
+      <c r="R13" s="109"/>
     </row>
     <row r="14" spans="1:18" ht="100.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A14" s="140"/>
-      <c r="B14" s="134"/>
-      <c r="C14" s="126" t="s">
+      <c r="A14" s="145"/>
+      <c r="B14" s="149"/>
+      <c r="C14" s="125" t="s">
         <v>56</v>
       </c>
-      <c r="D14" s="120" t="s">
+      <c r="D14" s="119" t="s">
         <v>62</v>
       </c>
-      <c r="E14" s="89"/>
-      <c r="F14" s="119" t="s">
+      <c r="E14" s="88"/>
+      <c r="F14" s="118" t="s">
         <v>22</v>
       </c>
-      <c r="G14" s="88" t="s">
+      <c r="G14" s="87" t="s">
         <v>32</v>
       </c>
-      <c r="H14" s="83" t="s">
+      <c r="H14" s="82" t="s">
         <v>32</v>
       </c>
-      <c r="I14" s="84" t="s">
+      <c r="I14" s="83" t="s">
         <v>32</v>
       </c>
-      <c r="L14" s="110"/>
-      <c r="M14" s="25"/>
-      <c r="N14" s="111"/>
-      <c r="O14" s="108"/>
-      <c r="P14" s="110"/>
-      <c r="Q14" s="108"/>
-      <c r="R14" s="110"/>
+      <c r="L14" s="109"/>
+      <c r="M14" s="24"/>
+      <c r="N14" s="110"/>
+      <c r="O14" s="107"/>
+      <c r="P14" s="109"/>
+      <c r="Q14" s="107"/>
+      <c r="R14" s="109"/>
     </row>
     <row r="15" spans="1:18" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="141">
+      <c r="A15" s="137">
         <f>A13 - 1</f>
         <v>9</v>
       </c>
-      <c r="B15" s="138" t="s">
+      <c r="B15" s="141" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="66">
+      <c r="C15" s="65">
         <f>I13 + 1</f>
         <v>3</v>
       </c>
-      <c r="D15" s="53">
+      <c r="D15" s="52">
         <f t="shared" ref="D15:I15" si="3">C15 + 1</f>
         <v>4</v>
       </c>
-      <c r="E15" s="82">
+      <c r="E15" s="81">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="F15" s="53">
+      <c r="F15" s="52">
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="G15" s="90">
+      <c r="G15" s="89">
         <f t="shared" si="3"/>
         <v>7</v>
       </c>
-      <c r="H15" s="54">
+      <c r="H15" s="53">
         <f t="shared" si="3"/>
         <v>8</v>
       </c>
-      <c r="I15" s="91">
+      <c r="I15" s="90">
         <f t="shared" si="3"/>
         <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:18" ht="103.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A16" s="142"/>
-      <c r="B16" s="137"/>
-      <c r="C16" s="85" t="s">
+      <c r="A16" s="138"/>
+      <c r="B16" s="142"/>
+      <c r="C16" s="84" t="s">
         <v>32</v>
       </c>
       <c r="D16" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="E16" s="63" t="s">
+      <c r="E16" s="62" t="s">
         <v>26</v>
       </c>
       <c r="F16" s="9" t="str">
@@ -2554,8 +2549,8 @@
 Team MS1 Prep
 (all in-class)</v>
       </c>
-      <c r="G16" s="92"/>
-      <c r="H16" s="63" t="str">
+      <c r="G16" s="91"/>
+      <c r="H16" s="62" t="str">
         <f>F16</f>
         <v>Team Session:
 Team Analysis &amp; Design Model
@@ -2563,69 +2558,69 @@
 Team MS1 Prep
 (all in-class)</v>
       </c>
-      <c r="I16" s="130" t="s">
+      <c r="I16" s="129" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:18" ht="6.4" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B17" s="24"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="25"/>
-      <c r="I17" s="25"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="24"/>
+      <c r="H17" s="24"/>
+      <c r="I17" s="24"/>
     </row>
     <row r="18" spans="1:18" ht="34.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B18" s="24"/>
-      <c r="C18" s="34" t="s">
+      <c r="B18" s="23"/>
+      <c r="C18" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="D18" s="72" t="s">
+      <c r="D18" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="E18" s="31" t="s">
+      <c r="E18" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="F18" s="32" t="s">
+      <c r="F18" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="G18" s="117" t="s">
+      <c r="G18" s="116" t="s">
         <v>43</v>
       </c>
-      <c r="H18" s="33" t="s">
+      <c r="H18" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="I18" s="62" t="s">
+      <c r="I18" s="61" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="19" spans="1:18" s="113" customFormat="1" ht="21.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A19" s="112"/>
-      <c r="B19" s="34"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="110"/>
-      <c r="E19" s="110"/>
-      <c r="F19" s="110"/>
-      <c r="G19" s="110"/>
-      <c r="H19" s="110"/>
-      <c r="I19" s="110"/>
+    <row r="19" spans="1:18" s="112" customFormat="1" ht="21.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A19" s="111"/>
+      <c r="B19" s="33"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="109"/>
+      <c r="E19" s="109"/>
+      <c r="F19" s="109"/>
+      <c r="G19" s="109"/>
+      <c r="H19" s="109"/>
+      <c r="I19" s="109"/>
     </row>
     <row r="20" spans="1:18" ht="54" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A20" s="149" t="str">
+      <c r="A20" s="132" t="str">
         <f>A1</f>
         <v>CS320: SW Engineering - Spring 2024 Schedule
-(as of 4-23-2024, subject to change)</v>
-      </c>
-      <c r="B20" s="150"/>
-      <c r="C20" s="150"/>
-      <c r="D20" s="150"/>
-      <c r="E20" s="150"/>
-      <c r="F20" s="150"/>
-      <c r="G20" s="150"/>
-      <c r="H20" s="150"/>
-      <c r="I20" s="151"/>
+(as of 5-5-2024, subject to change)</v>
+      </c>
+      <c r="B20" s="133"/>
+      <c r="C20" s="133"/>
+      <c r="D20" s="133"/>
+      <c r="E20" s="133"/>
+      <c r="F20" s="133"/>
+      <c r="G20" s="133"/>
+      <c r="H20" s="133"/>
+      <c r="I20" s="134"/>
     </row>
     <row r="21" spans="1:18" s="2" customFormat="1" ht="17.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A21" s="1" t="str">
@@ -2663,14 +2658,14 @@
       </c>
     </row>
     <row r="22" spans="1:18" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="152">
+      <c r="A22" s="135">
         <f>A15-1</f>
         <v>8</v>
       </c>
-      <c r="B22" s="138" t="s">
+      <c r="B22" s="141" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="93">
+      <c r="C22" s="92">
         <f>I15 + 1</f>
         <v>10</v>
       </c>
@@ -2698,44 +2693,44 @@
         <f t="shared" si="5"/>
         <v>16</v>
       </c>
-      <c r="L22" s="110"/>
-      <c r="M22" s="108"/>
-      <c r="N22" s="108"/>
-      <c r="O22" s="108"/>
-      <c r="P22" s="108"/>
-      <c r="Q22" s="108"/>
-      <c r="R22" s="108"/>
+      <c r="L22" s="109"/>
+      <c r="M22" s="107"/>
+      <c r="N22" s="107"/>
+      <c r="O22" s="107"/>
+      <c r="P22" s="107"/>
+      <c r="Q22" s="107"/>
+      <c r="R22" s="107"/>
     </row>
     <row r="23" spans="1:18" ht="67.150000000000006" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A23" s="145"/>
-      <c r="B23" s="138"/>
-      <c r="C23" s="131"/>
+      <c r="A23" s="136"/>
+      <c r="B23" s="141"/>
+      <c r="C23" s="130"/>
       <c r="D23" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="E23" s="54"/>
+      <c r="E23" s="53"/>
       <c r="F23" s="6" t="s">
         <v>63</v>
       </c>
       <c r="G23" s="6"/>
-      <c r="H23" s="22" t="s">
+      <c r="H23" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="I23" s="35"/>
-      <c r="L23" s="108"/>
-      <c r="M23" s="108"/>
-      <c r="N23" s="108"/>
-      <c r="O23" s="108"/>
-      <c r="P23" s="108"/>
-      <c r="Q23" s="108"/>
-      <c r="R23" s="25"/>
+      <c r="I23" s="34"/>
+      <c r="L23" s="107"/>
+      <c r="M23" s="107"/>
+      <c r="N23" s="107"/>
+      <c r="O23" s="107"/>
+      <c r="P23" s="107"/>
+      <c r="Q23" s="107"/>
+      <c r="R23" s="24"/>
     </row>
     <row r="24" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A24" s="145">
+      <c r="A24" s="136">
         <f>A22 - 1</f>
         <v>7</v>
       </c>
-      <c r="B24" s="138"/>
+      <c r="B24" s="141"/>
       <c r="C24" s="7">
         <f>I22 + 1</f>
         <v>17</v>
@@ -2764,44 +2759,44 @@
         <f t="shared" si="6"/>
         <v>23</v>
       </c>
-      <c r="L24" s="108"/>
-      <c r="M24" s="108"/>
-      <c r="N24" s="108"/>
-      <c r="O24" s="108"/>
-      <c r="P24" s="108"/>
-      <c r="Q24" s="108"/>
-      <c r="R24" s="108"/>
+      <c r="L24" s="107"/>
+      <c r="M24" s="107"/>
+      <c r="N24" s="107"/>
+      <c r="O24" s="107"/>
+      <c r="P24" s="107"/>
+      <c r="Q24" s="107"/>
+      <c r="R24" s="107"/>
     </row>
     <row r="25" spans="1:18" ht="124.15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="145"/>
-      <c r="B25" s="138"/>
-      <c r="C25" s="107"/>
-      <c r="D25" s="26" t="s">
+      <c r="A25" s="136"/>
+      <c r="B25" s="141"/>
+      <c r="C25" s="106"/>
+      <c r="D25" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="E25" s="124"/>
-      <c r="F25" s="54" t="s">
+      <c r="E25" s="123"/>
+      <c r="F25" s="53" t="s">
         <v>38</v>
       </c>
-      <c r="G25" s="124"/>
-      <c r="H25" s="132" t="s">
+      <c r="G25" s="123"/>
+      <c r="H25" s="131" t="s">
         <v>65</v>
       </c>
-      <c r="I25" s="128"/>
-      <c r="L25" s="25"/>
-      <c r="M25" s="108"/>
-      <c r="N25" s="110"/>
-      <c r="O25" s="108"/>
-      <c r="P25" s="110"/>
-      <c r="Q25" s="108"/>
-      <c r="R25" s="25"/>
+      <c r="I25" s="127"/>
+      <c r="L25" s="24"/>
+      <c r="M25" s="107"/>
+      <c r="N25" s="109"/>
+      <c r="O25" s="107"/>
+      <c r="P25" s="109"/>
+      <c r="Q25" s="107"/>
+      <c r="R25" s="24"/>
     </row>
     <row r="26" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A26" s="145">
+      <c r="A26" s="136">
         <f>A24 - 1</f>
         <v>6</v>
       </c>
-      <c r="B26" s="138"/>
+      <c r="B26" s="141"/>
       <c r="C26" s="7">
         <f>I24 + 1</f>
         <v>24</v>
@@ -2818,80 +2813,80 @@
         <f t="shared" si="7"/>
         <v>27</v>
       </c>
-      <c r="G26" s="80">
+      <c r="G26" s="79">
         <f t="shared" si="7"/>
         <v>28</v>
       </c>
-      <c r="H26" s="97">
+      <c r="H26" s="96">
         <f t="shared" ref="H26" si="8">G26 + 1</f>
         <v>29</v>
       </c>
-      <c r="I26" s="86">
+      <c r="I26" s="85">
         <f t="shared" ref="I26" si="9">H26 + 1</f>
         <v>30</v>
       </c>
-      <c r="L26" s="108"/>
-      <c r="M26" s="108"/>
-      <c r="N26" s="108"/>
-      <c r="O26" s="108"/>
-      <c r="P26" s="108"/>
-      <c r="Q26" s="108"/>
-      <c r="R26" s="108"/>
+      <c r="L26" s="107"/>
+      <c r="M26" s="107"/>
+      <c r="N26" s="107"/>
+      <c r="O26" s="107"/>
+      <c r="P26" s="107"/>
+      <c r="Q26" s="107"/>
+      <c r="R26" s="107"/>
     </row>
     <row r="27" spans="1:18" ht="68.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A27" s="142"/>
-      <c r="B27" s="137"/>
-      <c r="C27" s="127" t="s">
+      <c r="A27" s="138"/>
+      <c r="B27" s="142"/>
+      <c r="C27" s="126" t="s">
         <v>66</v>
       </c>
       <c r="D27" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="E27" s="54"/>
-      <c r="F27" s="23" t="s">
+      <c r="E27" s="53"/>
+      <c r="F27" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="G27" s="121" t="s">
+      <c r="G27" s="120" t="s">
         <v>41</v>
       </c>
-      <c r="H27" s="71" t="s">
+      <c r="H27" s="70" t="s">
         <v>36</v>
       </c>
-      <c r="I27" s="106" t="s">
+      <c r="I27" s="105" t="s">
         <v>36</v>
       </c>
-      <c r="L27" s="108"/>
-      <c r="M27" s="108"/>
-      <c r="N27" s="25"/>
-      <c r="O27" s="108"/>
-      <c r="P27" s="25"/>
-      <c r="Q27" s="110"/>
-      <c r="R27" s="25"/>
+      <c r="L27" s="107"/>
+      <c r="M27" s="107"/>
+      <c r="N27" s="24"/>
+      <c r="O27" s="107"/>
+      <c r="P27" s="24"/>
+      <c r="Q27" s="109"/>
+      <c r="R27" s="24"/>
     </row>
     <row r="28" spans="1:18" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A28" s="146">
+      <c r="A28" s="139">
         <f>A26 -1</f>
         <v>5</v>
       </c>
-      <c r="B28" s="133" t="s">
+      <c r="B28" s="143" t="s">
         <v>33</v>
       </c>
-      <c r="C28" s="98">
+      <c r="C28" s="97">
         <f>I26 + 1</f>
         <v>31</v>
       </c>
-      <c r="D28" s="99">
+      <c r="D28" s="98">
         <v>1</v>
       </c>
-      <c r="E28" s="39">
+      <c r="E28" s="38">
         <f t="shared" si="7"/>
         <v>2</v>
       </c>
-      <c r="F28" s="52">
+      <c r="F28" s="51">
         <f>E28 + 1</f>
         <v>3</v>
       </c>
-      <c r="G28" s="45">
+      <c r="G28" s="44">
         <f t="shared" si="7"/>
         <v>4</v>
       </c>
@@ -2899,47 +2894,47 @@
         <f>G28 + 1</f>
         <v>5</v>
       </c>
-      <c r="I28" s="58">
+      <c r="I28" s="57">
         <f>H28 + 1</f>
         <v>6</v>
       </c>
     </row>
     <row r="29" spans="1:18" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A29" s="147"/>
-      <c r="B29" s="134"/>
-      <c r="C29" s="116" t="s">
+      <c r="A29" s="150"/>
+      <c r="B29" s="149"/>
+      <c r="C29" s="115" t="s">
         <v>36</v>
       </c>
-      <c r="D29" s="100" t="s">
+      <c r="D29" s="99" t="s">
         <v>36</v>
       </c>
-      <c r="E29" s="50" t="s">
+      <c r="E29" s="49" t="s">
         <v>68</v>
       </c>
       <c r="F29" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="G29" s="50" t="s">
+      <c r="G29" s="49" t="s">
         <v>69</v>
       </c>
       <c r="H29" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="I29" s="28"/>
+      <c r="I29" s="27"/>
     </row>
     <row r="30" spans="1:18" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A30" s="148">
+      <c r="A30" s="151">
         <f>A28 -1</f>
         <v>4</v>
       </c>
-      <c r="B30" s="133" t="s">
+      <c r="B30" s="143" t="s">
         <v>13</v>
       </c>
-      <c r="C30" s="59">
+      <c r="C30" s="58">
         <f>I28 + 1</f>
         <v>7</v>
       </c>
-      <c r="D30" s="45">
+      <c r="D30" s="44">
         <f>C30 + 1</f>
         <v>8</v>
       </c>
@@ -2951,51 +2946,51 @@
         <f t="shared" si="10"/>
         <v>10</v>
       </c>
-      <c r="G30" s="45">
+      <c r="G30" s="44">
         <f t="shared" si="10"/>
         <v>11</v>
       </c>
-      <c r="H30" s="27">
+      <c r="H30" s="26">
         <f t="shared" si="10"/>
         <v>12</v>
       </c>
-      <c r="I30" s="28">
+      <c r="I30" s="27">
         <f t="shared" si="10"/>
         <v>13</v>
       </c>
     </row>
     <row r="31" spans="1:18" ht="87.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="139"/>
-      <c r="B31" s="135"/>
-      <c r="C31" s="30" t="s">
+      <c r="A31" s="140"/>
+      <c r="B31" s="144"/>
+      <c r="C31" s="29" t="s">
         <v>70</v>
       </c>
-      <c r="D31" s="104" t="s">
+      <c r="D31" s="103" t="s">
         <v>24</v>
       </c>
-      <c r="E31" s="105" t="s">
+      <c r="E31" s="104" t="s">
         <v>74</v>
       </c>
       <c r="F31" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="G31" s="27"/>
-      <c r="H31" s="27" t="s">
-        <v>75</v>
-      </c>
-      <c r="I31" s="28"/>
+      <c r="G31" s="26"/>
+      <c r="H31" s="26" t="s">
+        <v>81</v>
+      </c>
+      <c r="I31" s="27"/>
     </row>
     <row r="32" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A32" s="139">
+      <c r="A32" s="140">
         <f>A30 -1</f>
         <v>3</v>
       </c>
-      <c r="B32" s="135"/>
-      <c r="C32" s="27">
+      <c r="B32" s="144"/>
+      <c r="C32" s="26">
         <f>I30 + 1</f>
         <v>14</v>
       </c>
-      <c r="D32" s="27">
+      <c r="D32" s="26">
         <f>C32 + 1</f>
         <v>15</v>
       </c>
@@ -3007,47 +3002,47 @@
         <f t="shared" ref="F32:I32" si="11">E32 + 1</f>
         <v>17</v>
       </c>
-      <c r="G32" s="27">
+      <c r="G32" s="26">
         <f t="shared" si="11"/>
         <v>18</v>
       </c>
-      <c r="H32" s="27">
+      <c r="H32" s="26">
         <f t="shared" si="11"/>
         <v>19</v>
       </c>
-      <c r="I32" s="28">
+      <c r="I32" s="27">
         <f t="shared" si="11"/>
         <v>20</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" s="139"/>
-      <c r="B33" s="135"/>
-      <c r="C33" s="29"/>
-      <c r="D33" s="101" t="s">
+      <c r="A33" s="140"/>
+      <c r="B33" s="144"/>
+      <c r="C33" s="28"/>
+      <c r="D33" s="100" t="s">
         <v>6</v>
       </c>
       <c r="E33" s="11"/>
-      <c r="F33" s="44" t="s">
+      <c r="F33" s="43" t="s">
         <v>71</v>
       </c>
-      <c r="G33" s="78"/>
+      <c r="G33" s="77"/>
       <c r="H33" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="I33" s="28"/>
+      <c r="I33" s="27"/>
     </row>
     <row r="34" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A34" s="139">
+      <c r="A34" s="140">
         <f>A32 -1</f>
         <v>2</v>
       </c>
-      <c r="B34" s="135"/>
-      <c r="C34" s="29">
+      <c r="B34" s="144"/>
+      <c r="C34" s="28">
         <f>I32 + 1</f>
         <v>21</v>
       </c>
-      <c r="D34" s="27">
+      <c r="D34" s="26">
         <f>C34 + 1</f>
         <v>22</v>
       </c>
@@ -3073,28 +3068,28 @@
       </c>
     </row>
     <row r="35" spans="1:9" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A35" s="140"/>
-      <c r="B35" s="134"/>
-      <c r="C35" s="57"/>
-      <c r="D35" s="43" t="s">
+      <c r="A35" s="145"/>
+      <c r="B35" s="149"/>
+      <c r="C35" s="56"/>
+      <c r="D35" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="E35" s="42"/>
-      <c r="F35" s="44" t="s">
-        <v>77</v>
-      </c>
-      <c r="G35" s="42"/>
-      <c r="H35" s="155" t="s">
+      <c r="E35" s="41"/>
+      <c r="F35" s="43" t="s">
+        <v>75</v>
+      </c>
+      <c r="G35" s="41"/>
+      <c r="H35" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="I35" s="41"/>
+      <c r="I35" s="40"/>
     </row>
     <row r="36" spans="1:9" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A36" s="141">
+      <c r="A36" s="137">
         <f>A34 -1</f>
         <v>1</v>
       </c>
-      <c r="B36" s="136" t="s">
+      <c r="B36" s="146" t="s">
         <v>34</v>
       </c>
       <c r="C36" s="17">
@@ -3109,7 +3104,7 @@
         <f t="shared" si="12"/>
         <v>30</v>
       </c>
-      <c r="F36" s="94">
+      <c r="F36" s="93">
         <v>1</v>
       </c>
       <c r="G36" s="4">
@@ -3126,29 +3121,29 @@
       </c>
     </row>
     <row r="37" spans="1:9" ht="85.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A37" s="142"/>
-      <c r="B37" s="137"/>
-      <c r="C37" s="60" t="s">
-        <v>80</v>
-      </c>
-      <c r="D37" s="49" t="s">
+      <c r="A37" s="138"/>
+      <c r="B37" s="142"/>
+      <c r="C37" s="59" t="s">
+        <v>78</v>
+      </c>
+      <c r="D37" s="48" t="s">
         <v>6</v>
       </c>
-      <c r="E37" s="96"/>
-      <c r="F37" s="95" t="s">
+      <c r="E37" s="95"/>
+      <c r="F37" s="94" t="s">
         <v>6</v>
       </c>
       <c r="G37" s="6"/>
       <c r="H37" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="I37" s="91"/>
+      <c r="I37" s="90"/>
     </row>
     <row r="38" spans="1:9" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A38" s="143" t="s">
+      <c r="A38" s="152" t="s">
         <v>25</v>
       </c>
-      <c r="B38" s="138" t="s">
+      <c r="B38" s="141" t="s">
         <v>5</v>
       </c>
       <c r="C38" s="20">
@@ -3159,7 +3154,7 @@
         <f t="shared" ref="D38:I38" si="13">C38 + 1</f>
         <v>6</v>
       </c>
-      <c r="E38" s="55">
+      <c r="E38" s="54">
         <f t="shared" si="13"/>
         <v>7</v>
       </c>
@@ -3171,35 +3166,47 @@
         <f t="shared" si="13"/>
         <v>9</v>
       </c>
-      <c r="H38" s="73">
+      <c r="H38" s="72">
         <f t="shared" si="13"/>
         <v>10</v>
       </c>
-      <c r="I38" s="74">
+      <c r="I38" s="73">
         <f t="shared" si="13"/>
         <v>11</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="103.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A39" s="144"/>
-      <c r="B39" s="137"/>
-      <c r="C39" s="156" t="s">
-        <v>81</v>
-      </c>
-      <c r="D39" s="23" t="s">
-        <v>78</v>
-      </c>
-      <c r="E39" s="61"/>
-      <c r="F39" s="23" t="s">
-        <v>79</v>
-      </c>
-      <c r="G39" s="21"/>
-      <c r="H39" s="75"/>
-      <c r="I39" s="76"/>
+      <c r="A39" s="153"/>
+      <c r="B39" s="142"/>
+      <c r="C39" s="154"/>
+      <c r="D39" s="22" t="s">
+        <v>76</v>
+      </c>
+      <c r="E39" s="60"/>
+      <c r="F39" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="G39" s="124" t="s">
+        <v>80</v>
+      </c>
+      <c r="H39" s="74"/>
+      <c r="I39" s="75"/>
     </row>
     <row r="40" spans="1:9" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="B30:B35"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="A32:A33"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A22:A23"/>
     <mergeCell ref="A3:A4"/>
@@ -3216,18 +3223,6 @@
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="B13:B14"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="A30:A31"/>
-    <mergeCell ref="A32:A33"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="B30:B35"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="A36:A37"/>
-    <mergeCell ref="A38:A39"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0" footer="0"/>

</xml_diff>